<commit_message>
Sync tracker with Week 1 completion
Week 1 is fully done after PR #5 merge — flip 9 Week 1 rows from
Not Started to Done and add evidence links. Overall progress now
38/98 (38.8%). Also refresh the stale Week 0 deliverable note that
referenced the deleted week0_bootstrap.ipynb.
</commit_message>
<xml_diff>
--- a/docs/bharatgen_intern_tracker.xlsx
+++ b/docs/bharatgen_intern_tracker.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="655" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deliverables" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cadence" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Success Criteria" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anti-Patterns" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Learning Resources" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tracker" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Glossary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Deliverables" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Cadence" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Success Criteria" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Anti-Patterns" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Learning Resources" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tracker'!$A$1:$J$99</definedName>
@@ -593,7 +593,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="21" t="inlineStr">
         <is>
@@ -684,7 +683,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="21" t="inlineStr">
         <is>
@@ -700,7 +698,6 @@
       </c>
     </row>
     <row r="14"/>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="21" t="inlineStr">
         <is>
@@ -1964,7 +1961,7 @@
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>Consolidated 60-cell bootstrap notebook + reflection.md (NN, training, why-data, GD, backprop, attention/transformers) committed</t>
+          <t>Per-day notebooks (day1_numpy, day2_matplotlib_librosa, day3_ml_tokens_tensor, day5_pytorch_tensors) + reflection.md (NN, training, attention/transformers) committed. Intern split the single bootstrap notebook by day; deliverable spec accepted as 'Done'.</t>
         </is>
       </c>
     </row>
@@ -2232,11 +2229,19 @@
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I32" s="7" t="n"/>
-      <c r="J32" s="7" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I32" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/blob/claude/setup-intern-project-FkRbX/week1/week1_audio_basics.ipynb</t>
+        </is>
+      </c>
+      <c r="J32" s="7" t="inlineStr">
+        <is>
+          <t>Covered in week1_audio_basics.ipynb + mel-spec plots for 5 languages</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="61.5" customHeight="1">
       <c r="A33" s="7" t="inlineStr">
@@ -2275,11 +2280,19 @@
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I33" s="7" t="n"/>
-      <c r="J33" s="7" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/blob/claude/setup-intern-project-FkRbX/week1/week1_tensors_matmul.ipynb</t>
+        </is>
+      </c>
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t>.shape/.dtype/.device/.to()/.numpy() walked through with examples</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="61.5" customHeight="1">
       <c r="A34" s="7" t="inlineStr">
@@ -2318,11 +2331,19 @@
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I34" s="7" t="n"/>
-      <c r="J34" s="7" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I34" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/claude/setup-intern-project-FkRbX/week1/data/audio_clips</t>
+        </is>
+      </c>
+      <c r="J34" s="7" t="inlineStr">
+        <is>
+          <t>5 .wav clips committed: English, Hindi, Kannada, Marathi, Telugu</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="61.5" customHeight="1">
       <c r="A35" s="7" t="inlineStr">
@@ -2361,11 +2382,19 @@
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I35" s="7" t="n"/>
-      <c r="J35" s="7" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/claude/setup-intern-project-FkRbX/week1/data/plots</t>
+        </is>
+      </c>
+      <c r="J35" s="7" t="inlineStr">
+        <is>
+          <t>Side-by-side waveform + mel-spectrogram PNGs for all 5 language clips</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="61.5" customHeight="1">
       <c r="A36" s="7" t="inlineStr">
@@ -2404,11 +2433,19 @@
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I36" s="7" t="n"/>
-      <c r="J36" s="7" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I36" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/blob/claude/setup-intern-project-FkRbX/week1/resampling_16khz.ipynb</t>
+        </is>
+      </c>
+      <c r="J36" s="7" t="inlineStr">
+        <is>
+          <t>48kHz-&gt;16kHz torchaudio resample with subjective listen-comparison notes</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="61.5" customHeight="1">
       <c r="A37" s="7" t="inlineStr">
@@ -2447,11 +2484,19 @@
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I37" s="7" t="n"/>
-      <c r="J37" s="7" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/blob/claude/setup-intern-project-FkRbX/week1/week1_tensors_matmul.ipynb</t>
+        </is>
+      </c>
+      <c r="J37" s="7" t="inlineStr">
+        <is>
+          <t>Benchmarks at 1000/2500/10000 matrix sizes, CPU vs GPU with synchronize()</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="61.5" customHeight="1">
       <c r="A38" s="7" t="inlineStr">
@@ -2490,11 +2535,19 @@
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I38" s="7" t="n"/>
-      <c r="J38" s="7" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/claude/setup-intern-project-FkRbX/week1</t>
+        </is>
+      </c>
+      <c r="J38" s="7" t="inlineStr">
+        <is>
+          <t>Both deliverable files present: week1_audio_basics.ipynb and audio_cheatsheet.md</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="61.5" customHeight="1">
       <c r="A39" s="7" t="inlineStr">
@@ -2533,11 +2586,15 @@
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I39" s="7" t="n"/>
-      <c r="J39" s="7" t="n"/>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>No detour into CS224S — stayed on librosa/torchaudio primitives</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="61.5" customHeight="1">
       <c r="A40" s="7" t="inlineStr">
@@ -2576,11 +2633,15 @@
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I40" s="7" t="n"/>
-      <c r="J40" s="7" t="n"/>
+      <c r="J40" s="7" t="inlineStr">
+        <is>
+          <t>Used librosa/torch primitives directly; no FFT re-derivation</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="61.5" customHeight="1">
       <c r="A41" s="7" t="inlineStr">
@@ -6412,10 +6473,14 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/claude/setup-intern-project-FkRbX/week1</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="63.75" customHeight="1">
       <c r="A4" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Sync tracker with Week 2 deliverable (Done with caveats)
PR #7 lands the Week 2 HF mental-model artifacts. Marking all 11 items
Done; deliverable flagged "Done (with caveats)" with the gaps captured
in row notes (no pipeline-vs-manual comparison, no cache screenshot,
no GPU/device cell, model.eval() not invoked, prose typos). Full
review on the PR.
</commit_message>
<xml_diff>
--- a/docs/bharatgen_intern_tracker.xlsx
+++ b/docs/bharatgen_intern_tracker.xlsx
@@ -2680,11 +2680,19 @@
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I41" s="7" t="n"/>
-      <c r="J41" s="7" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/week2/week2/how_to_run_an_hf_model.md</t>
+        </is>
+      </c>
+      <c r="J41" s="7" t="inlineStr">
+        <is>
+          <t>Auto* classes explained in how_to_run_an_hf_model.md; used across distilbert_manual.ipynb and whisper-tiny.ipynb</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="61.5" customHeight="1">
       <c r="A42" s="7" t="inlineStr">
@@ -2723,11 +2731,19 @@
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I42" s="7" t="n"/>
-      <c r="J42" s="7" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I42" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/week2/week2/how_to_run_an_hf_model.md</t>
+        </is>
+      </c>
+      <c r="J42" s="7" t="inlineStr">
+        <is>
+          <t>trust_remote_code section in how_to_run_an_hf_model.md covers the security implication</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="61.5" customHeight="1">
       <c r="A43" s="7" t="inlineStr">
@@ -2766,11 +2782,19 @@
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I43" s="7" t="n"/>
-      <c r="J43" s="7" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I43" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/week2/week2/distilbert_manual.ipynb</t>
+        </is>
+      </c>
+      <c r="J43" s="7" t="inlineStr">
+        <is>
+          <t>Both concepts in tutorial; torch.no_grad() used in distilbert_manual.ipynb. Caveat: model.eval() explained but not invoked in the manual notebook</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="61.5" customHeight="1">
       <c r="A44" s="7" t="inlineStr">
@@ -2809,11 +2833,19 @@
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I44" s="7" t="n"/>
-      <c r="J44" s="7" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I44" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/week2/week2/distilbert_manual.ipynb</t>
+        </is>
+      </c>
+      <c r="J44" s="7" t="inlineStr">
+        <is>
+          <t>Logits printed and softmax applied manually in distilbert_manual.ipynb</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="61.5" customHeight="1">
       <c r="A45" s="7" t="inlineStr">
@@ -2852,11 +2884,19 @@
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I45" s="7" t="n"/>
-      <c r="J45" s="7" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I45" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/week2/week2/how_to_run_an_hf_model.md</t>
+        </is>
+      </c>
+      <c r="J45" s="7" t="inlineStr">
+        <is>
+          <t>Cache behavior described in tutorial. Caveat: spec asked for a screenshot of the cache dir — missing</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="61.5" customHeight="1">
       <c r="A46" s="7" t="inlineStr">
@@ -2895,11 +2935,19 @@
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I46" s="7" t="n"/>
-      <c r="J46" s="7" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I46" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/week2/week2/distilbert_manual.ipynb</t>
+        </is>
+      </c>
+      <c r="J46" s="7" t="inlineStr">
+        <is>
+          <t>Manual AutoTokenizer+AutoModel path with logits+softmax. Caveat: pipeline() side-by-side comparison missing — spec asked for it</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="61.5" customHeight="1">
       <c r="A47" s="7" t="inlineStr">
@@ -2938,11 +2986,19 @@
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I47" s="7" t="n"/>
-      <c r="J47" s="7" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I47" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/week2/week2/whisper-tiny.ipynb</t>
+        </is>
+      </c>
+      <c r="J47" s="7" t="inlineStr">
+        <is>
+          <t>whisper-tiny run on all 5 Week 1 clips; transcripts in whisper_tiny_baseline.json. Note: Indic outputs are largely hallucinated — expected for tiny, becomes the Week 3 baseline</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="61.5" customHeight="1">
       <c r="A48" s="7" t="inlineStr">
@@ -2981,11 +3037,19 @@
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I48" s="7" t="n"/>
-      <c r="J48" s="7" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I48" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/week2/week2/how_to_run_an_hf_model.md</t>
+        </is>
+      </c>
+      <c r="J48" s="7" t="inlineStr">
+        <is>
+          <t>hidden_size / num_hidden_layers / vocab_size explained in plain English in tutorial</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="61.5" customHeight="1">
       <c r="A49" s="7" t="inlineStr">
@@ -3024,11 +3088,19 @@
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I49" s="7" t="n"/>
-      <c r="J49" s="7" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I49" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/week2/week2/how_to_run_an_hf_model.md</t>
+        </is>
+      </c>
+      <c r="J49" s="7" t="inlineStr">
+        <is>
+          <t>PR #7 (week2 -&gt; claude/setup-intern-project-FkRbX). Done with caveats: (1) no pipeline()-vs-manual comparison, (2) no cache screenshot, (3) no GPU/device cell, (4) prose typos. See PR review for full list</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="61.5" customHeight="1">
       <c r="A50" s="7" t="inlineStr">
@@ -3067,11 +3139,15 @@
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I50" s="7" t="n"/>
-      <c r="J50" s="7" t="n"/>
+      <c r="J50" s="7" t="inlineStr">
+        <is>
+          <t>No fine-tuning attempted in Week 2 artifacts</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="61.5" customHeight="1">
       <c r="A51" s="7" t="inlineStr">
@@ -3110,11 +3186,15 @@
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I51" s="7" t="n"/>
-      <c r="J51" s="7" t="n"/>
+      <c r="J51" s="7" t="inlineStr">
+        <is>
+          <t>No accelerate/bitsandbytes/vLLM pulled in Week 2 artifacts</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="61.5" customHeight="1">
       <c r="A52" s="7" t="inlineStr">
@@ -6505,10 +6585,14 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="n"/>
+          <t>Done (with caveats)</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/pull/7</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="63.75" customHeight="1">
       <c r="A5" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Point Week 2 tracker evidence at the default branch
Following the Week 1 convention. The week2 feature branch may be
deleted later; default-branch URLs survive that.
</commit_message>
<xml_diff>
--- a/docs/bharatgen_intern_tracker.xlsx
+++ b/docs/bharatgen_intern_tracker.xlsx
@@ -2685,7 +2685,7 @@
       </c>
       <c r="I41" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/week2/week2/how_to_run_an_hf_model.md</t>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/claude/setup-intern-project-FkRbX/week2/how_to_run_an_hf_model.md</t>
         </is>
       </c>
       <c r="J41" s="7" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="I42" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/week2/week2/how_to_run_an_hf_model.md</t>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/claude/setup-intern-project-FkRbX/week2/how_to_run_an_hf_model.md</t>
         </is>
       </c>
       <c r="J42" s="7" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="I43" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/week2/week2/distilbert_manual.ipynb</t>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/claude/setup-intern-project-FkRbX/week2/distilbert_manual.ipynb</t>
         </is>
       </c>
       <c r="J43" s="7" t="inlineStr">
@@ -2838,7 +2838,7 @@
       </c>
       <c r="I44" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/week2/week2/distilbert_manual.ipynb</t>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/claude/setup-intern-project-FkRbX/week2/distilbert_manual.ipynb</t>
         </is>
       </c>
       <c r="J44" s="7" t="inlineStr">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="I45" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/week2/week2/how_to_run_an_hf_model.md</t>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/claude/setup-intern-project-FkRbX/week2/how_to_run_an_hf_model.md</t>
         </is>
       </c>
       <c r="J45" s="7" t="inlineStr">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="I46" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/week2/week2/distilbert_manual.ipynb</t>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/claude/setup-intern-project-FkRbX/week2/distilbert_manual.ipynb</t>
         </is>
       </c>
       <c r="J46" s="7" t="inlineStr">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="I47" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/week2/week2/whisper-tiny.ipynb</t>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/claude/setup-intern-project-FkRbX/week2/whisper-tiny.ipynb</t>
         </is>
       </c>
       <c r="J47" s="7" t="inlineStr">
@@ -3042,7 +3042,7 @@
       </c>
       <c r="I48" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/week2/week2/how_to_run_an_hf_model.md</t>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/claude/setup-intern-project-FkRbX/week2/how_to_run_an_hf_model.md</t>
         </is>
       </c>
       <c r="J48" s="7" t="inlineStr">
@@ -3093,7 +3093,7 @@
       </c>
       <c r="I49" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/week2/week2/how_to_run_an_hf_model.md</t>
+          <t>https://github.com/makarkul/bharatgen-speech-intern-2026/tree/claude/setup-intern-project-FkRbX/week2/how_to_run_an_hf_model.md</t>
         </is>
       </c>
       <c r="J49" s="7" t="inlineStr">

</xml_diff>